<commit_message>
Last edits befor revise
</commit_message>
<xml_diff>
--- a/Results/Sit_To_Stand/Normal/FindPrincipalComponents_PipelinePCA_Sit_To_Stand/PCA_Dimension_Search_PipelinePCA.xlsx
+++ b/Results/Sit_To_Stand/Normal/FindPrincipalComponents_PipelinePCA_Sit_To_Stand/PCA_Dimension_Search_PipelinePCA.xlsx
@@ -1202,40 +1202,40 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>80</v>
+        <v>78.66666666666667</v>
       </c>
       <c r="C14" t="n">
-        <v>83.5925925925926</v>
+        <v>82.57671957671958</v>
       </c>
       <c r="D14" t="n">
-        <v>80</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="E14" t="n">
-        <v>90</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="F14" t="n">
-        <v>79.35257335257336</v>
+        <v>78.12025012025011</v>
       </c>
       <c r="G14" t="n">
-        <v>80</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="H14" t="n">
-        <v>5.962847939999443</v>
+        <v>4.988876515698592</v>
       </c>
       <c r="I14" t="n">
-        <v>5.74683070049372</v>
+        <v>5.137443532993981</v>
       </c>
       <c r="J14" t="n">
-        <v>5.962847939999437</v>
+        <v>4.988876515698586</v>
       </c>
       <c r="K14" t="n">
-        <v>2.981423969999714</v>
+        <v>2.49443825784929</v>
       </c>
       <c r="L14" t="n">
-        <v>6.08950358915116</v>
+        <v>5.267247944321596</v>
       </c>
       <c r="M14" t="n">
-        <v>5.962847939999437</v>
+        <v>4.988876515698586</v>
       </c>
     </row>
     <row r="15">
@@ -1612,40 +1612,40 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>77.33333333333333</v>
+        <v>78.66666666666667</v>
       </c>
       <c r="C24" t="n">
-        <v>80.9047619047619</v>
+        <v>81.53968253968256</v>
       </c>
       <c r="D24" t="n">
-        <v>77.33333333333333</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="E24" t="n">
-        <v>88.66666666666667</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="F24" t="n">
-        <v>77.02993302993303</v>
+        <v>78.62444962444964</v>
       </c>
       <c r="G24" t="n">
-        <v>77.33333333333333</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="H24" t="n">
-        <v>8.000000000000004</v>
+        <v>7.774602526460404</v>
       </c>
       <c r="I24" t="n">
-        <v>7.266582759020995</v>
+        <v>7.312207597201438</v>
       </c>
       <c r="J24" t="n">
-        <v>8.000000000000002</v>
+        <v>7.774602526460401</v>
       </c>
       <c r="K24" t="n">
-        <v>3.999999999999994</v>
+        <v>3.887301263230194</v>
       </c>
       <c r="L24" t="n">
-        <v>8.260257441202528</v>
+        <v>7.810187934648827</v>
       </c>
       <c r="M24" t="n">
-        <v>8.000000000000002</v>
+        <v>7.774602526460401</v>
       </c>
     </row>
     <row r="25">
@@ -1694,28 +1694,28 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>76</v>
+        <v>77.33333333333333</v>
       </c>
       <c r="C26" t="n">
-        <v>79.71428571428571</v>
+        <v>80.34920634920636</v>
       </c>
       <c r="D26" t="n">
-        <v>76</v>
+        <v>77.33333333333331</v>
       </c>
       <c r="E26" t="n">
-        <v>87.99999999999999</v>
+        <v>88.66666666666664</v>
       </c>
       <c r="F26" t="n">
-        <v>75.51478151478152</v>
+        <v>77.10929810929811</v>
       </c>
       <c r="G26" t="n">
-        <v>76</v>
+        <v>77.33333333333331</v>
       </c>
       <c r="H26" t="n">
-        <v>9.043106644167025</v>
+        <v>9.043106644167027</v>
       </c>
       <c r="I26" t="n">
-        <v>8.670445132498472</v>
+        <v>8.795083259638069</v>
       </c>
       <c r="J26" t="n">
         <v>9.043106644167025</v>
@@ -1724,7 +1724,7 @@
         <v>4.521553322083506</v>
       </c>
       <c r="L26" t="n">
-        <v>9.446088563166928</v>
+        <v>9.318135016784074</v>
       </c>
       <c r="M26" t="n">
         <v>9.043106644167025</v>
@@ -1817,40 +1817,40 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>80</v>
+        <v>78.66666666666667</v>
       </c>
       <c r="C29" t="n">
-        <v>83.42857142857143</v>
+        <v>82.53968253968254</v>
       </c>
       <c r="D29" t="n">
-        <v>80</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="E29" t="n">
-        <v>90</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="F29" t="n">
-        <v>79.9072779072779</v>
+        <v>78.49650349650349</v>
       </c>
       <c r="G29" t="n">
-        <v>80</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="H29" t="n">
-        <v>7.302967433402217</v>
+        <v>6.53197264742181</v>
       </c>
       <c r="I29" t="n">
-        <v>6.231932817875243</v>
+        <v>5.853679020503421</v>
       </c>
       <c r="J29" t="n">
-        <v>7.302967433402217</v>
+        <v>6.53197264742181</v>
       </c>
       <c r="K29" t="n">
-        <v>3.651483716701103</v>
+        <v>3.2659863237109</v>
       </c>
       <c r="L29" t="n">
-        <v>7.313557785221052</v>
+        <v>6.524363810315431</v>
       </c>
       <c r="M29" t="n">
-        <v>7.302967433402217</v>
+        <v>6.53197264742181</v>
       </c>
     </row>
     <row r="30">
@@ -1899,28 +1899,28 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>77.33333333333333</v>
+        <v>76</v>
       </c>
       <c r="C31" t="n">
-        <v>80.34920634920636</v>
+        <v>79.71428571428571</v>
       </c>
       <c r="D31" t="n">
-        <v>77.33333333333331</v>
+        <v>76</v>
       </c>
       <c r="E31" t="n">
-        <v>88.66666666666664</v>
+        <v>87.99999999999999</v>
       </c>
       <c r="F31" t="n">
-        <v>77.10929810929811</v>
+        <v>75.51478151478152</v>
       </c>
       <c r="G31" t="n">
-        <v>77.33333333333331</v>
+        <v>76</v>
       </c>
       <c r="H31" t="n">
-        <v>9.043106644167027</v>
+        <v>9.043106644167025</v>
       </c>
       <c r="I31" t="n">
-        <v>8.795083259638069</v>
+        <v>8.670445132498472</v>
       </c>
       <c r="J31" t="n">
         <v>9.043106644167025</v>
@@ -1929,7 +1929,7 @@
         <v>4.521553322083506</v>
       </c>
       <c r="L31" t="n">
-        <v>9.318135016784074</v>
+        <v>9.446088563166928</v>
       </c>
       <c r="M31" t="n">
         <v>9.043106644167025</v>
@@ -1940,40 +1940,40 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>78.66666666666667</v>
+        <v>77.33333333333333</v>
       </c>
       <c r="C32" t="n">
-        <v>82.7936507936508</v>
+        <v>80.34920634920636</v>
       </c>
       <c r="D32" t="n">
-        <v>78.66666666666666</v>
+        <v>77.33333333333331</v>
       </c>
       <c r="E32" t="n">
-        <v>89.33333333333333</v>
+        <v>88.66666666666664</v>
       </c>
       <c r="F32" t="n">
-        <v>78.31276131276131</v>
+        <v>77.10929810929811</v>
       </c>
       <c r="G32" t="n">
-        <v>78.66666666666666</v>
+        <v>77.33333333333331</v>
       </c>
       <c r="H32" t="n">
-        <v>7.774602526460404</v>
+        <v>9.043106644167027</v>
       </c>
       <c r="I32" t="n">
-        <v>6.369491405198453</v>
+        <v>8.795083259638069</v>
       </c>
       <c r="J32" t="n">
-        <v>7.774602526460401</v>
+        <v>9.043106644167025</v>
       </c>
       <c r="K32" t="n">
-        <v>3.887301263230194</v>
+        <v>4.521553322083506</v>
       </c>
       <c r="L32" t="n">
-        <v>8.050585498455682</v>
+        <v>9.318135016784074</v>
       </c>
       <c r="M32" t="n">
-        <v>7.774602526460401</v>
+        <v>9.043106644167025</v>
       </c>
     </row>
     <row r="33">
@@ -1981,40 +1981,40 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>78.66666666666667</v>
+        <v>77.33333333333333</v>
       </c>
       <c r="C33" t="n">
-        <v>81.53968253968256</v>
+        <v>80.34920634920636</v>
       </c>
       <c r="D33" t="n">
-        <v>78.66666666666666</v>
+        <v>77.33333333333331</v>
       </c>
       <c r="E33" t="n">
-        <v>89.33333333333333</v>
+        <v>88.66666666666664</v>
       </c>
       <c r="F33" t="n">
-        <v>78.62444962444964</v>
+        <v>77.10929810929811</v>
       </c>
       <c r="G33" t="n">
-        <v>78.66666666666666</v>
+        <v>77.33333333333331</v>
       </c>
       <c r="H33" t="n">
-        <v>7.774602526460404</v>
+        <v>9.043106644167027</v>
       </c>
       <c r="I33" t="n">
-        <v>7.312207597201438</v>
+        <v>8.795083259638069</v>
       </c>
       <c r="J33" t="n">
-        <v>7.774602526460401</v>
+        <v>9.043106644167025</v>
       </c>
       <c r="K33" t="n">
-        <v>3.887301263230194</v>
+        <v>4.521553322083506</v>
       </c>
       <c r="L33" t="n">
-        <v>7.810187934648827</v>
+        <v>9.318135016784074</v>
       </c>
       <c r="M33" t="n">
-        <v>7.774602526460401</v>
+        <v>9.043106644167025</v>
       </c>
     </row>
     <row r="34">
@@ -2145,40 +2145,40 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>78.66666666666667</v>
+        <v>80</v>
       </c>
       <c r="C37" t="n">
-        <v>81.53968253968256</v>
+        <v>83.42857142857143</v>
       </c>
       <c r="D37" t="n">
-        <v>78.66666666666666</v>
+        <v>80</v>
       </c>
       <c r="E37" t="n">
-        <v>89.33333333333333</v>
+        <v>90</v>
       </c>
       <c r="F37" t="n">
-        <v>78.62444962444964</v>
+        <v>79.9072779072779</v>
       </c>
       <c r="G37" t="n">
-        <v>78.66666666666666</v>
+        <v>80</v>
       </c>
       <c r="H37" t="n">
-        <v>7.774602526460404</v>
+        <v>7.302967433402217</v>
       </c>
       <c r="I37" t="n">
-        <v>7.312207597201438</v>
+        <v>6.231932817875243</v>
       </c>
       <c r="J37" t="n">
-        <v>7.774602526460401</v>
+        <v>7.302967433402217</v>
       </c>
       <c r="K37" t="n">
-        <v>3.887301263230194</v>
+        <v>3.651483716701103</v>
       </c>
       <c r="L37" t="n">
-        <v>7.810187934648827</v>
+        <v>7.313557785221052</v>
       </c>
       <c r="M37" t="n">
-        <v>7.774602526460401</v>
+        <v>7.302967433402217</v>
       </c>
     </row>
     <row r="38">
@@ -2186,40 +2186,40 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>77.33333333333333</v>
+        <v>78.66666666666667</v>
       </c>
       <c r="C38" t="n">
-        <v>80.34920634920636</v>
+        <v>81.53968253968256</v>
       </c>
       <c r="D38" t="n">
-        <v>77.33333333333331</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="E38" t="n">
-        <v>88.66666666666664</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="F38" t="n">
-        <v>77.10929810929811</v>
+        <v>78.62444962444964</v>
       </c>
       <c r="G38" t="n">
-        <v>77.33333333333331</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="H38" t="n">
-        <v>9.043106644167027</v>
+        <v>7.774602526460404</v>
       </c>
       <c r="I38" t="n">
-        <v>8.795083259638069</v>
+        <v>7.312207597201438</v>
       </c>
       <c r="J38" t="n">
-        <v>9.043106644167025</v>
+        <v>7.774602526460401</v>
       </c>
       <c r="K38" t="n">
-        <v>4.521553322083506</v>
+        <v>3.887301263230194</v>
       </c>
       <c r="L38" t="n">
-        <v>9.318135016784074</v>
+        <v>7.810187934648827</v>
       </c>
       <c r="M38" t="n">
-        <v>9.043106644167025</v>
+        <v>7.774602526460401</v>
       </c>
     </row>
     <row r="39">
@@ -2309,40 +2309,40 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>77.33333333333333</v>
+        <v>78.66666666666667</v>
       </c>
       <c r="C41" t="n">
-        <v>80.34920634920636</v>
+        <v>81.53968253968256</v>
       </c>
       <c r="D41" t="n">
-        <v>77.33333333333331</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="E41" t="n">
-        <v>88.66666666666664</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="F41" t="n">
-        <v>77.10929810929811</v>
+        <v>78.62444962444964</v>
       </c>
       <c r="G41" t="n">
-        <v>77.33333333333331</v>
+        <v>78.66666666666666</v>
       </c>
       <c r="H41" t="n">
-        <v>9.043106644167027</v>
+        <v>7.774602526460404</v>
       </c>
       <c r="I41" t="n">
-        <v>8.795083259638069</v>
+        <v>7.312207597201438</v>
       </c>
       <c r="J41" t="n">
-        <v>9.043106644167025</v>
+        <v>7.774602526460401</v>
       </c>
       <c r="K41" t="n">
-        <v>4.521553322083506</v>
+        <v>3.887301263230194</v>
       </c>
       <c r="L41" t="n">
-        <v>9.318135016784074</v>
+        <v>7.810187934648827</v>
       </c>
       <c r="M41" t="n">
-        <v>9.043106644167025</v>
+        <v>7.774602526460401</v>
       </c>
     </row>
     <row r="42">
@@ -2514,40 +2514,40 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>78.66666666666667</v>
+        <v>77.33333333333333</v>
       </c>
       <c r="C46" t="n">
-        <v>81.53968253968256</v>
+        <v>80.34920634920636</v>
       </c>
       <c r="D46" t="n">
-        <v>78.66666666666666</v>
+        <v>77.33333333333331</v>
       </c>
       <c r="E46" t="n">
-        <v>89.33333333333333</v>
+        <v>88.66666666666664</v>
       </c>
       <c r="F46" t="n">
-        <v>78.62444962444964</v>
+        <v>77.10929810929811</v>
       </c>
       <c r="G46" t="n">
-        <v>78.66666666666666</v>
+        <v>77.33333333333331</v>
       </c>
       <c r="H46" t="n">
-        <v>7.774602526460404</v>
+        <v>9.043106644167027</v>
       </c>
       <c r="I46" t="n">
-        <v>7.312207597201438</v>
+        <v>8.795083259638069</v>
       </c>
       <c r="J46" t="n">
-        <v>7.774602526460401</v>
+        <v>9.043106644167025</v>
       </c>
       <c r="K46" t="n">
-        <v>3.887301263230194</v>
+        <v>4.521553322083506</v>
       </c>
       <c r="L46" t="n">
-        <v>7.810187934648827</v>
+        <v>9.318135016784074</v>
       </c>
       <c r="M46" t="n">
-        <v>7.774602526460401</v>
+        <v>9.043106644167025</v>
       </c>
     </row>
     <row r="47">
@@ -4390,22 +4390,22 @@
         <v>3</v>
       </c>
       <c r="C64" t="n">
-        <v>86.66666666666667</v>
+        <v>80</v>
       </c>
       <c r="D64" t="n">
-        <v>88.8888888888889</v>
+        <v>83.80952380952381</v>
       </c>
       <c r="E64" t="n">
-        <v>86.66666666666667</v>
+        <v>80</v>
       </c>
       <c r="F64" t="n">
-        <v>93.33333333333333</v>
+        <v>90</v>
       </c>
       <c r="G64" t="n">
-        <v>85.60606060606061</v>
+        <v>79.44444444444444</v>
       </c>
       <c r="H64" t="n">
-        <v>86.66666666666667</v>
+        <v>80</v>
       </c>
     </row>
     <row r="65">
@@ -5664,22 +5664,22 @@
         <v>2</v>
       </c>
       <c r="C113" t="n">
-        <v>73.33333333333333</v>
+        <v>80</v>
       </c>
       <c r="D113" t="n">
-        <v>80.15873015873015</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="E113" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="F113" t="n">
-        <v>86.66666666666667</v>
+        <v>90</v>
       </c>
       <c r="G113" t="n">
-        <v>71.57287157287158</v>
+        <v>79.54545454545455</v>
       </c>
       <c r="H113" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
     </row>
     <row r="114">
@@ -5924,22 +5924,22 @@
         <v>2</v>
       </c>
       <c r="C123" t="n">
-        <v>73.33333333333333</v>
+        <v>80</v>
       </c>
       <c r="D123" t="n">
-        <v>80.15873015873015</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="E123" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="F123" t="n">
-        <v>86.66666666666667</v>
+        <v>90</v>
       </c>
       <c r="G123" t="n">
-        <v>71.57287157287158</v>
+        <v>79.54545454545455</v>
       </c>
       <c r="H123" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
     </row>
     <row r="124">
@@ -6366,22 +6366,22 @@
         <v>4</v>
       </c>
       <c r="C140" t="n">
-        <v>86.66666666666667</v>
+        <v>80</v>
       </c>
       <c r="D140" t="n">
-        <v>87.77777777777777</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="E140" t="n">
-        <v>86.66666666666667</v>
+        <v>80</v>
       </c>
       <c r="F140" t="n">
-        <v>93.33333333333333</v>
+        <v>90</v>
       </c>
       <c r="G140" t="n">
-        <v>86.5993265993266</v>
+        <v>79.54545454545455</v>
       </c>
       <c r="H140" t="n">
-        <v>86.66666666666667</v>
+        <v>80</v>
       </c>
     </row>
     <row r="141">
@@ -6574,22 +6574,22 @@
         <v>2</v>
       </c>
       <c r="C148" t="n">
-        <v>80</v>
+        <v>73.33333333333333</v>
       </c>
       <c r="D148" t="n">
-        <v>83.33333333333334</v>
+        <v>80.15873015873015</v>
       </c>
       <c r="E148" t="n">
-        <v>80</v>
+        <v>73.33333333333334</v>
       </c>
       <c r="F148" t="n">
-        <v>90</v>
+        <v>86.66666666666667</v>
       </c>
       <c r="G148" t="n">
-        <v>79.54545454545455</v>
+        <v>71.57287157287158</v>
       </c>
       <c r="H148" t="n">
-        <v>80</v>
+        <v>73.33333333333334</v>
       </c>
     </row>
     <row r="149">
@@ -6782,22 +6782,22 @@
         <v>5</v>
       </c>
       <c r="C156" t="n">
-        <v>73.33333333333333</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="D156" t="n">
-        <v>80.15873015873015</v>
+        <v>67.93650793650792</v>
       </c>
       <c r="E156" t="n">
-        <v>73.33333333333334</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="F156" t="n">
-        <v>86.66666666666667</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="G156" t="n">
-        <v>71.57287157287158</v>
+        <v>65.55555555555556</v>
       </c>
       <c r="H156" t="n">
-        <v>73.33333333333334</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="157">
@@ -6912,22 +6912,22 @@
         <v>5</v>
       </c>
       <c r="C161" t="n">
-        <v>73.33333333333333</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="D161" t="n">
-        <v>73.88888888888889</v>
+        <v>67.93650793650792</v>
       </c>
       <c r="E161" t="n">
-        <v>73.33333333333334</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="F161" t="n">
-        <v>86.66666666666667</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="G161" t="n">
-        <v>73.13131313131315</v>
+        <v>65.55555555555556</v>
       </c>
       <c r="H161" t="n">
-        <v>73.33333333333334</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="162">
@@ -7432,22 +7432,22 @@
         <v>5</v>
       </c>
       <c r="C181" t="n">
-        <v>73.33333333333333</v>
+        <v>80</v>
       </c>
       <c r="D181" t="n">
-        <v>73.88888888888889</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="E181" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="F181" t="n">
-        <v>86.66666666666667</v>
+        <v>90</v>
       </c>
       <c r="G181" t="n">
-        <v>73.13131313131315</v>
+        <v>79.54545454545455</v>
       </c>
       <c r="H181" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
     </row>
     <row r="182">
@@ -7562,22 +7562,22 @@
         <v>5</v>
       </c>
       <c r="C186" t="n">
-        <v>66.66666666666666</v>
+        <v>73.33333333333333</v>
       </c>
       <c r="D186" t="n">
-        <v>67.93650793650792</v>
+        <v>73.88888888888889</v>
       </c>
       <c r="E186" t="n">
-        <v>66.66666666666666</v>
+        <v>73.33333333333334</v>
       </c>
       <c r="F186" t="n">
-        <v>83.33333333333334</v>
+        <v>86.66666666666667</v>
       </c>
       <c r="G186" t="n">
-        <v>65.55555555555556</v>
+        <v>73.13131313131315</v>
       </c>
       <c r="H186" t="n">
-        <v>66.66666666666666</v>
+        <v>73.33333333333334</v>
       </c>
     </row>
     <row r="187">
@@ -7952,22 +7952,22 @@
         <v>5</v>
       </c>
       <c r="C201" t="n">
-        <v>66.66666666666666</v>
+        <v>73.33333333333333</v>
       </c>
       <c r="D201" t="n">
-        <v>67.93650793650792</v>
+        <v>73.88888888888889</v>
       </c>
       <c r="E201" t="n">
-        <v>66.66666666666666</v>
+        <v>73.33333333333334</v>
       </c>
       <c r="F201" t="n">
-        <v>83.33333333333334</v>
+        <v>86.66666666666667</v>
       </c>
       <c r="G201" t="n">
-        <v>65.55555555555556</v>
+        <v>73.13131313131315</v>
       </c>
       <c r="H201" t="n">
-        <v>66.66666666666666</v>
+        <v>73.33333333333334</v>
       </c>
     </row>
     <row r="202">
@@ -8602,22 +8602,22 @@
         <v>5</v>
       </c>
       <c r="C226" t="n">
-        <v>73.33333333333333</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="D226" t="n">
-        <v>73.88888888888889</v>
+        <v>67.93650793650792</v>
       </c>
       <c r="E226" t="n">
-        <v>73.33333333333334</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="F226" t="n">
-        <v>86.66666666666667</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="G226" t="n">
-        <v>73.13131313131315</v>
+        <v>65.55555555555556</v>
       </c>
       <c r="H226" t="n">
-        <v>73.33333333333334</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="227">

</xml_diff>